<commit_message>
YHAAO-5343 update basic info template
</commit_message>
<xml_diff>
--- a/src/src/main/resources/template/APM_Asset_Dynamic_Template_en.xlsx
+++ b/src/src/main/resources/template/APM_Asset_Dynamic_Template_en.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\503156711\IdeaProjects\hc-apm-web\src\src\main\resources\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9912B3B7-505C-4B1E-A437-ADFDA72A79A1}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F10DA42-A679-45C2-B2F2-B3A44382287C}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-18210" yWindow="5415" windowWidth="22425" windowHeight="12885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Asset List" sheetId="2" r:id="rId1"/>
     <sheet name="Org List" sheetId="11" r:id="rId2"/>
     <sheet name="User List" sheetId="9" state="hidden" r:id="rId3"/>
-    <sheet name="必填字段检查表" sheetId="15" r:id="rId4"/>
-    <sheet name="必填字段填写说明" sheetId="14" r:id="rId5"/>
+    <sheet name="Required field checklist" sheetId="15" r:id="rId4"/>
+    <sheet name="Required fields to fill in the " sheetId="14" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Org List'!$4:$4</definedName>
@@ -60,20 +60,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="108">
-  <si>
-    <t>设备列表</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="105">
   <si>
     <t>人员列表</t>
   </si>
   <si>
-    <t>部门列表</t>
-  </si>
-  <si>
-    <t>部门名称</t>
-  </si>
-  <si>
     <t>人员编号</t>
   </si>
   <si>
@@ -86,22 +77,10 @@
     <t>李四</t>
   </si>
   <si>
-    <t>总价值</t>
-  </si>
-  <si>
     <t>医院代号</t>
   </si>
   <si>
     <t>人员名字</t>
-  </si>
-  <si>
-    <t>生产日期</t>
-  </si>
-  <si>
-    <t>安装日期</t>
-  </si>
-  <si>
-    <t>功能分组</t>
   </si>
   <si>
     <t>医院名称</t>
@@ -126,24 +105,12 @@
 所有日期格式为MM/DD/YYYY</t>
   </si>
   <si>
-    <t>字段</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>系统强制性必填</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>实施要求必填</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>Y</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>M</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -161,6 +128,171 @@
     </r>
   </si>
   <si>
+    <t>S</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>M</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>S</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>M</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>S</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>v2.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment ID </t>
+  </si>
+  <si>
+    <t>Equipment Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment Alias </t>
+  </si>
+  <si>
+    <t>Repair Owner</t>
+  </si>
+  <si>
+    <t>Repair Owner 2</t>
+  </si>
+  <si>
+    <t>Manufacturer</t>
+  </si>
+  <si>
+    <t>Registration Number</t>
+  </si>
+  <si>
+    <t>Vendor</t>
+  </si>
+  <si>
+    <t>Equipment Classification</t>
+  </si>
+  <si>
+    <t>Function Grade</t>
+  </si>
+  <si>
+    <t>Equipment Model</t>
+  </si>
+  <si>
+    <t>Manufacturer Serial Number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">System ID/Manufacturer Request ID </t>
+  </si>
+  <si>
+    <t>Asset ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bar Code </t>
+  </si>
+  <si>
+    <t xml:space="preserve">IT System ID </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Purchase Price </t>
+  </si>
+  <si>
+    <t>Final Salvage Value</t>
+  </si>
+  <si>
+    <t>Depreciation Method</t>
+  </si>
+  <si>
+    <t>Life Cycle</t>
+  </si>
+  <si>
+    <t>Purchase Date</t>
+  </si>
+  <si>
+    <t>Arrival Date</t>
+  </si>
+  <si>
+    <t>Warranty Expiration Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terminate Date </t>
+  </si>
+  <si>
+    <t>Last Maintenance Date</t>
+  </si>
+  <si>
+    <t>Last Measurement Date</t>
+  </si>
+  <si>
+    <t>Last Inspection Date</t>
+  </si>
+  <si>
+    <t>Maintainer</t>
+  </si>
+  <si>
+    <t>Maintainer Telephone</t>
+  </si>
+  <si>
+    <t>QR Code</t>
+  </si>
+  <si>
+    <t>Legend</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Check Item</t>
+  </si>
+  <si>
+    <t>Device List</t>
+  </si>
+  <si>
+    <t>Template file version number</t>
+  </si>
+  <si>
+    <t>All date formats are MM/DD/YYYY</t>
+  </si>
+  <si>
+    <t>The total number</t>
+  </si>
+  <si>
+    <t>total value</t>
+  </si>
+  <si>
+    <t>Department list</t>
+  </si>
+  <si>
+    <t>Department name</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Required or not</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>Implementation requirements are required</t>
+  </si>
+  <si>
+    <t>System mandatory</t>
+  </si>
+  <si>
+    <t>Suggested, otherwise the function will be limited</t>
+  </si>
+  <si>
     <r>
       <t>1</t>
     </r>
@@ -172,7 +304,7 @@
         <family val="3"/>
         <charset val="134"/>
       </rPr>
-      <t>，自动派工必填；</t>
+      <t>，Automatic dispatch must be filled；</t>
     </r>
     <r>
       <rPr>
@@ -192,17 +324,7 @@
         <family val="3"/>
         <charset val="134"/>
       </rPr>
-      <t>，</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color indexed="63"/>
-        <rFont val="Franklin Gothic Medium"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>用途：推消息</t>
+      <t>，Purpose: tweet messages</t>
     </r>
     <r>
       <rPr>
@@ -216,97 +338,92 @@
     </r>
   </si>
   <si>
-    <t>使用部门</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>S</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>目前可自由输入，将来要求必填</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>M</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>S</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>M</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>Y</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>S</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>建议填，否则功能会受限制</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>系统完全必填检查项</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>是否满足</t>
-  </si>
-  <si>
-    <t>说明</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>设备名称是否已填写</t>
-  </si>
-  <si>
-    <t>必须有有效数据</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>实施必填检查项</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>维修负责人是否已填写</t>
-  </si>
-  <si>
-    <t>维修负责人的名字是否已在系统中建立</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>使用部门是否已填写</t>
-  </si>
-  <si>
-    <t>注册证号是否已填写</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>功能分组是否已填写</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>设备型号是否已填写</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>SystemID/厂商报修ID是否全部已填写</t>
-  </si>
-  <si>
-    <t>资产编号是否已填写</t>
-  </si>
-  <si>
-    <t>对于大放设备，IT系统编号是否已填写</t>
+    <t>At present, it is free to enter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">user department </t>
+  </si>
+  <si>
+    <t>date of manufacture</t>
+  </si>
+  <si>
+    <t>Functional groups</t>
+  </si>
+  <si>
+    <t xml:space="preserve">installation date </t>
+  </si>
+  <si>
+    <t>The system must complete the check item</t>
+  </si>
+  <si>
+    <t>whether it satisfies</t>
+  </si>
+  <si>
+    <t>Has the device number been filled in</t>
+  </si>
+  <si>
+    <t>There must be valid data and no duplication</t>
+  </si>
+  <si>
+    <t>Has the device name been filled in</t>
+  </si>
+  <si>
+    <t>Whether the equipment classification has been filled in</t>
+  </si>
+  <si>
+    <t>There must be valid data</t>
+  </si>
+  <si>
+    <t>Implement mandatory check items</t>
+  </si>
+  <si>
+    <t xml:space="preserve">explain </t>
+  </si>
+  <si>
+    <t>Has the maintenance supervisor filled in</t>
+  </si>
+  <si>
+    <t>Is the maintenance manager's name established in the system</t>
+  </si>
+  <si>
+    <t>Whether the using department has been filled in</t>
+  </si>
+  <si>
+    <t>Has the registration number been filled in</t>
+  </si>
+  <si>
+    <t>Whether the function group has been filled in</t>
+  </si>
+  <si>
+    <t>Has the device model been filled in</t>
+  </si>
+  <si>
+    <t>Whether all SystemID/ the repair ID of the manufacturer has been filled in</t>
+  </si>
+  <si>
+    <t>Whether the asset number has been filled in</t>
+  </si>
+  <si>
+    <t>For large storage equipment, whether the IT system number has been filled in</t>
+  </si>
+  <si>
+    <t>Has the installation date been entered</t>
+  </si>
+  <si>
+    <t>Whether the expiry date of maintenance has been filled in</t>
+  </si>
+  <si>
+    <t>Whether the qr code has been filled in</t>
+  </si>
+  <si>
+    <t>Whether the qr code has no duplicate value</t>
+  </si>
+  <si>
+    <t>Whether the qr code will be automatically adjusted by Excel</t>
   </si>
   <si>
     <r>
-      <t>RIS</t>
+      <t>The RIS</t>
     </r>
     <r>
       <rPr>
@@ -316,192 +433,23 @@
         <family val="3"/>
         <charset val="134"/>
       </rPr>
-      <t>集成版必须填写</t>
+      <t xml:space="preserve"> integration version must be filled in</t>
     </r>
   </si>
   <si>
-    <t>安装日期是否已填写</t>
-  </si>
-  <si>
-    <t>维保截止日期是否已填写</t>
-  </si>
-  <si>
-    <t>二维码是否已填写</t>
-  </si>
-  <si>
-    <t>二维码是否没有重复值</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>二维码是否会被Excel自动调整格式</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>建议填写检查项</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>设备编号是否已填写</t>
-  </si>
-  <si>
-    <t>必须有有效数据</t>
-  </si>
-  <si>
-    <t>设备编号是否不重复</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>制造商是否已填写</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>建议尽量填，否则功能会受限制</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>采购价格是否已填写</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>必须有有效数据且院区不重复</t>
-  </si>
-  <si>
-    <r>
-      <t>所有日期格式为</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Franklin Gothic Medium"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>MM/DD/YYYY</t>
-    </r>
-  </si>
-  <si>
-    <t>模版文件版本号</t>
-  </si>
-  <si>
-    <t>v2.4</t>
-  </si>
-  <si>
-    <t>设备分类是否已填写</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equipment ID </t>
-  </si>
-  <si>
-    <t>Equipment Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equipment Alias </t>
-  </si>
-  <si>
-    <t>Repair Owner</t>
-  </si>
-  <si>
-    <t>Repair Owner 2</t>
-  </si>
-  <si>
-    <t>Manufacturer</t>
-  </si>
-  <si>
-    <t>Registration Number</t>
-  </si>
-  <si>
-    <t>Vendor</t>
-  </si>
-  <si>
-    <t>Equipment Classification</t>
-  </si>
-  <si>
-    <t>Function Grade</t>
-  </si>
-  <si>
-    <t>Equipment Model</t>
-  </si>
-  <si>
-    <t>Manufacturer Serial Number</t>
-  </si>
-  <si>
-    <t xml:space="preserve">System ID/Manufacturer Request ID </t>
-  </si>
-  <si>
-    <t>Asset ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bar Code </t>
-  </si>
-  <si>
-    <t xml:space="preserve">IT System ID </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Purchase Price </t>
-  </si>
-  <si>
-    <t>Final Salvage Value</t>
-  </si>
-  <si>
-    <t>Depreciation Method</t>
-  </si>
-  <si>
-    <t>Life Cycle</t>
-  </si>
-  <si>
-    <t>Purchase Date</t>
-  </si>
-  <si>
-    <t>Arrival Date</t>
-  </si>
-  <si>
-    <t>Warranty Expiration Date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Terminate Date </t>
-  </si>
-  <si>
-    <t>Last Maintenance Date</t>
-  </si>
-  <si>
-    <t>Last Measurement Date</t>
-  </si>
-  <si>
-    <t>Last Inspection Date</t>
-  </si>
-  <si>
-    <t>Maintainer</t>
-  </si>
-  <si>
-    <t>Maintainer Telephone</t>
-  </si>
-  <si>
-    <t>QR Code</t>
-  </si>
-  <si>
-    <t>是否必填</t>
-  </si>
-  <si>
-    <t>注释</t>
-  </si>
-  <si>
-    <t>Legend</t>
-  </si>
-  <si>
-    <t>系统强制性必填</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Check Item</t>
-  </si>
-  <si>
-    <t>说明</t>
-  </si>
-  <si>
-    <t>总数量</t>
+    <t>It is suggested to fill in the check item</t>
+  </si>
+  <si>
+    <t>Whether the device number is not repeated</t>
+  </si>
+  <si>
+    <t>Whether the manufacturer has filled in</t>
+  </si>
+  <si>
+    <t>Has the purchase price been filled in</t>
+  </si>
+  <si>
+    <t>It is recommended to fill in as many as possible, otherwise the function will be limited</t>
   </si>
 </sst>
 </file>
@@ -514,10 +462,17 @@
     <numFmt numFmtId="165" formatCode="&quot;&quot;;&quot;&quot;;&quot;Clear Pick List Selected in B2&quot;"/>
     <numFmt numFmtId="166" formatCode="[$¥-804]#,##0.00"/>
   </numFmts>
-  <fonts count="37">
+  <fonts count="38">
     <font>
       <sz val="11"/>
       <color theme="3" tint="0.14993743705557422"/>
+      <name val="Franklin Gothic Medium"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Franklin Gothic Medium"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1121,288 +1076,288 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0">
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="7" fontId="4" fillId="0" borderId="0">
+    <xf numFmtId="7" fontId="5" fillId="0" borderId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="12" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="4"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="12"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="4" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="12" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="12" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="4"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="12"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="4" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="12" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="7">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="7">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="10">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="10">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="10" applyFont="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="10" applyFont="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="10" applyFill="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="10" applyFill="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="10" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="10" applyFont="1" applyFill="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="4" borderId="3" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="4" borderId="3" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="4" xfId="14" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="23" fillId="0" borderId="4" xfId="14" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="22" fillId="0" borderId="4" xfId="14" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="23" fillId="0" borderId="4" xfId="14" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="7" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="7" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="25" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="15"/>
-    <xf numFmtId="0" fontId="29" fillId="9" borderId="6" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="15"/>
+    <xf numFmtId="0" fontId="30" fillId="9" borderId="6" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="9" borderId="7" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="9" borderId="7" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="8" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="4" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="4" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="9" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="10" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="11" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="11" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="12" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="15" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="15" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="16" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="17" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="18" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="18" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="19" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="4" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="4" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="9" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="9" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="11" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="11" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="12" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="15" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="7" borderId="15" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="12" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="15" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="8" borderId="15" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="7" borderId="16" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="8" borderId="16" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="17" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="18" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="18" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="19" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="4" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="9" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="11" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="12" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="15" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="8" borderId="15" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="20" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="21" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="15" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="15" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="12" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="12" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="37" fillId="4" borderId="3" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="5" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="8" borderId="16" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="7" borderId="13" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="20" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="21" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="15" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="15" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="15" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="15" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="12" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="12" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="4" borderId="3" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="9" borderId="5" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="7" borderId="14" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="7" borderId="13" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="7" borderId="7" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="7" borderId="14" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="13" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="7" borderId="7" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="14" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="8" borderId="13" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="7" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="8" borderId="14" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="8" borderId="7" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="15" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="15" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="16">
     <cellStyle name="Flag Column" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -1604,7 +1559,7 @@
         <a:p>
           <a:pPr marL="0" indent="0" algn="ctr"/>
           <a:r>
-            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
+            <a:rPr lang="en-US" sz="1100">
               <a:solidFill>
                 <a:schemeClr val="lt1"/>
               </a:solidFill>
@@ -1612,16 +1567,8 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>部门列表</a:t>
+            <a:t>Department list</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:schemeClr val="lt1"/>
-            </a:solidFill>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -1701,7 +1648,7 @@
         <a:p>
           <a:pPr marL="0" indent="0" algn="ctr"/>
           <a:r>
-            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
+            <a:rPr lang="en-US" sz="1100">
               <a:solidFill>
                 <a:schemeClr val="lt1"/>
               </a:solidFill>
@@ -1709,16 +1656,8 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>设备列表</a:t>
+            <a:t>Device List</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:schemeClr val="lt1"/>
-            </a:solidFill>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -2076,21 +2015,21 @@
     <col min="3" max="3" width="10.08984375" customWidth="1"/>
     <col min="4" max="4" width="11.453125" customWidth="1"/>
     <col min="5" max="5" width="13.453125" customWidth="1"/>
-    <col min="6" max="8" width="13.453125" style="71" customWidth="1"/>
+    <col min="6" max="8" width="13.453125" style="69" customWidth="1"/>
     <col min="9" max="9" width="17.08984375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.31640625" style="71" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.31640625" style="71" customWidth="1"/>
+    <col min="10" max="10" width="16.31640625" style="69" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.31640625" style="69" customWidth="1"/>
     <col min="12" max="12" width="9.08984375" customWidth="1"/>
-    <col min="13" max="13" width="18.76953125" style="74" customWidth="1"/>
+    <col min="13" max="13" width="18.76953125" style="72" customWidth="1"/>
     <col min="14" max="14" width="22.453125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="24.6796875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="19" customWidth="1"/>
-    <col min="17" max="17" width="19" style="71" customWidth="1"/>
+    <col min="17" max="17" width="19" style="69" customWidth="1"/>
     <col min="18" max="18" width="10" customWidth="1"/>
-    <col min="19" max="19" width="10" style="71" customWidth="1"/>
+    <col min="19" max="19" width="10" style="69" customWidth="1"/>
     <col min="20" max="21" width="10.08984375" customWidth="1"/>
     <col min="22" max="22" width="19.08984375" customWidth="1"/>
-    <col min="23" max="23" width="19.08984375" style="71" customWidth="1"/>
+    <col min="23" max="23" width="19.08984375" style="69" customWidth="1"/>
     <col min="24" max="24" width="14.6796875" customWidth="1"/>
     <col min="25" max="26" width="10.08984375" customWidth="1"/>
     <col min="27" max="27" width="13.6796875" customWidth="1"/>
@@ -2101,23 +2040,23 @@
     <col min="32" max="32" width="11.453125" customWidth="1"/>
     <col min="33" max="33" width="10.08984375" customWidth="1"/>
     <col min="34" max="34" width="11.453125" customWidth="1"/>
-    <col min="35" max="35" width="11.453125" style="71" customWidth="1"/>
+    <col min="35" max="35" width="11.453125" style="69" customWidth="1"/>
     <col min="36" max="36" width="13.08984375" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="13.31640625" customWidth="1"/>
     <col min="38" max="38" width="14.6796875" customWidth="1"/>
     <col min="39" max="39" width="12.453125" customWidth="1"/>
     <col min="40" max="40" width="12.6796875" customWidth="1"/>
-    <col min="41" max="42" width="12.31640625" style="74" customWidth="1"/>
-    <col min="43" max="43" width="16.08984375" style="74" customWidth="1"/>
-    <col min="44" max="44" width="12.76953125" style="74" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="9.08984375" style="74" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="11.08984375" style="74" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="9.08984375" style="74" bestFit="1" customWidth="1"/>
+    <col min="41" max="42" width="12.31640625" style="72" customWidth="1"/>
+    <col min="43" max="43" width="16.08984375" style="72" customWidth="1"/>
+    <col min="44" max="44" width="12.76953125" style="72" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="9.08984375" style="72" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="11.08984375" style="72" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="9.08984375" style="72" bestFit="1" customWidth="1"/>
     <col min="51" max="51" width="9.31640625" bestFit="1" customWidth="1"/>
     <col min="52" max="52" width="11.6796875" customWidth="1"/>
     <col min="53" max="54" width="12.76953125" bestFit="1" customWidth="1"/>
     <col min="55" max="55" width="11.31640625" customWidth="1"/>
-    <col min="56" max="57" width="11.31640625" style="71" customWidth="1"/>
+    <col min="56" max="57" width="11.31640625" style="69" customWidth="1"/>
     <col min="58" max="58" width="27.453125" customWidth="1"/>
     <col min="59" max="59" width="10.76953125" bestFit="1" customWidth="1"/>
     <col min="60" max="60" width="11.6796875" bestFit="1" customWidth="1"/>
@@ -2126,51 +2065,51 @@
   <sheetData>
     <row r="1" spans="1:69" ht="27" hidden="1" customHeight="1">
       <c r="A1" s="14" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C1" s="14"/>
-      <c r="D1" s="75" t="s">
-        <v>20</v>
-      </c>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="76"/>
-      <c r="K1" s="76"/>
-      <c r="L1" s="76"/>
-      <c r="M1" s="76"/>
-      <c r="BG1" s="76"/>
-    </row>
-    <row r="2" spans="1:69" ht="13.8">
-      <c r="A2" s="77"/>
-      <c r="B2" s="79" t="s">
-        <v>67</v>
+      <c r="D1" s="73" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="74"/>
+      <c r="F1" s="74"/>
+      <c r="G1" s="74"/>
+      <c r="H1" s="74"/>
+      <c r="I1" s="74"/>
+      <c r="J1" s="74"/>
+      <c r="K1" s="74"/>
+      <c r="L1" s="74"/>
+      <c r="M1" s="74"/>
+      <c r="BG1" s="74"/>
+    </row>
+    <row r="2" spans="1:69" ht="24.6">
+      <c r="A2" s="75"/>
+      <c r="B2" s="77" t="s">
+        <v>58</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="D2" s="76"/>
-      <c r="E2" s="78" t="s">
-        <v>66</v>
-      </c>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="76"/>
-      <c r="I2" s="76"/>
-      <c r="J2" s="76"/>
-      <c r="K2" s="76"/>
-      <c r="L2" s="76"/>
-      <c r="M2" s="76"/>
-      <c r="BG2" s="76"/>
+        <v>23</v>
+      </c>
+      <c r="D2" s="74"/>
+      <c r="E2" s="76" t="s">
+        <v>59</v>
+      </c>
+      <c r="F2" s="74"/>
+      <c r="G2" s="74"/>
+      <c r="H2" s="74"/>
+      <c r="I2" s="74"/>
+      <c r="J2" s="74"/>
+      <c r="K2" s="74"/>
+      <c r="L2" s="74"/>
+      <c r="M2" s="74"/>
+      <c r="BG2" s="74"/>
     </row>
     <row r="3" spans="1:69" ht="34.799999999999997" thickBot="1">
       <c r="A3" s="5" t="s">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -2180,20 +2119,20 @@
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
       <c r="I3" s="1"/>
-      <c r="J3" s="72"/>
-      <c r="K3" s="72"/>
+      <c r="J3" s="70"/>
+      <c r="K3" s="70"/>
       <c r="L3" s="1"/>
-      <c r="M3" s="73"/>
+      <c r="M3" s="71"/>
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
       <c r="P3" s="1"/>
-      <c r="Q3" s="72"/>
+      <c r="Q3" s="70"/>
       <c r="R3" s="1"/>
-      <c r="S3" s="72"/>
+      <c r="S3" s="70"/>
       <c r="T3" s="1"/>
       <c r="U3" s="1"/>
       <c r="V3" s="1"/>
-      <c r="W3" s="72"/>
+      <c r="W3" s="70"/>
       <c r="X3" s="1"/>
       <c r="Y3" s="1"/>
       <c r="Z3" s="1"/>
@@ -2205,19 +2144,19 @@
       <c r="AF3" s="1"/>
       <c r="AG3" s="1"/>
       <c r="AH3" s="1"/>
-      <c r="AI3" s="72"/>
+      <c r="AI3" s="70"/>
       <c r="AJ3" s="1"/>
       <c r="AK3" s="1"/>
       <c r="AL3" s="1"/>
       <c r="AM3" s="1"/>
       <c r="AN3" s="1"/>
-      <c r="AO3" s="73"/>
-      <c r="AP3" s="73"/>
-      <c r="AQ3" s="73"/>
-      <c r="AR3" s="73"/>
-      <c r="AS3" s="73"/>
-      <c r="AT3" s="73"/>
-      <c r="AU3" s="73"/>
+      <c r="AO3" s="71"/>
+      <c r="AP3" s="71"/>
+      <c r="AQ3" s="71"/>
+      <c r="AR3" s="71"/>
+      <c r="AS3" s="71"/>
+      <c r="AT3" s="71"/>
+      <c r="AU3" s="71"/>
       <c r="AV3" s="1"/>
       <c r="AW3" s="1"/>
       <c r="AX3" s="1"/>
@@ -2225,28 +2164,28 @@
       <c r="AZ3" s="1"/>
       <c r="BA3" s="1"/>
       <c r="BB3" s="1"/>
-      <c r="BC3" s="72"/>
-      <c r="BD3" s="72"/>
-      <c r="BE3" s="72"/>
-      <c r="BF3" s="72"/>
+      <c r="BC3" s="70"/>
+      <c r="BD3" s="70"/>
+      <c r="BE3" s="70"/>
+      <c r="BF3" s="70"/>
       <c r="BG3" s="1"/>
-      <c r="BH3" s="72"/>
-      <c r="BI3" s="72"/>
-      <c r="BJ3" s="72"/>
-      <c r="BK3" s="72"/>
-      <c r="BL3" s="72"/>
-      <c r="BM3" s="72"/>
-      <c r="BN3" s="72"/>
-      <c r="BO3" s="72"/>
-      <c r="BP3" s="72"/>
-      <c r="BQ3" s="72"/>
+      <c r="BH3" s="70"/>
+      <c r="BI3" s="70"/>
+      <c r="BJ3" s="70"/>
+      <c r="BK3" s="70"/>
+      <c r="BL3" s="70"/>
+      <c r="BM3" s="70"/>
+      <c r="BN3" s="70"/>
+      <c r="BO3" s="70"/>
+      <c r="BP3" s="70"/>
+      <c r="BQ3" s="70"/>
     </row>
     <row r="4" spans="1:69" ht="13.8">
       <c r="A4" s="2" t="s">
-        <v>107</v>
+        <v>60</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>8</v>
+        <v>61</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="2"/>
@@ -2259,7 +2198,7 @@
       <c r="BI4" s="8"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="18" type="noConversion"/>
+  <phoneticPr fontId="19" type="noConversion"/>
   <conditionalFormatting sqref="D1 E4:H4">
     <cfRule type="expression" dxfId="4" priority="85">
       <formula>"If(blnBinNo=""True"")"</formula>
@@ -2299,7 +2238,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="34.799999999999997" thickBot="1">
       <c r="A1" s="5" t="s">
-        <v>2</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:1">
@@ -2309,12 +2248,12 @@
       <c r="A3" s="11"/>
     </row>
     <row r="4" spans="1:1">
-      <c r="A4" s="80" t="s">
-        <v>3</v>
+      <c r="A4" s="78" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="18" type="noConversion"/>
+  <phoneticPr fontId="19" type="noConversion"/>
   <dataValidations xWindow="567" yWindow="330" count="1">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="To clear the pick list table in this worksheet, activate the object in B2 or press ALT+F8 and type &quot;ClearPickList&quot; with no spaces, then select RUN" sqref="A2" xr:uid="{00000000-0002-0000-0100-000000000000}"/>
   </dataValidations>
@@ -2344,7 +2283,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="34.799999999999997" thickBot="1">
       <c r="A1" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2361,24 +2300,24 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="10" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B5" s="10">
         <v>1</v>
@@ -2387,15 +2326,15 @@
         <v>18900000000</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="10" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B6" s="10">
         <v>2</v>
@@ -2404,10 +2343,10 @@
         <v>18911111111</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -2617,7 +2556,7 @@
       <c r="D39" s="12"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="18" type="noConversion"/>
+  <phoneticPr fontId="19" type="noConversion"/>
   <dataValidations xWindow="144" yWindow="400" count="2">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Navigation link to Warehouse Inventory List worksheet" sqref="A2" xr:uid="{00000000-0002-0000-0200-000000000000}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5:D8" xr:uid="{00000000-0002-0000-0200-000001000000}">
@@ -2651,25 +2590,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A1" s="81" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="81"/>
-      <c r="D1" s="81"/>
+      <c r="A1" s="79" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
     </row>
     <row r="2" spans="1:4" ht="15.6" thickBot="1">
       <c r="A2" s="36" t="s">
-        <v>104</v>
+        <v>55</v>
       </c>
       <c r="B2" s="37" t="s">
-        <v>105</v>
+        <v>56</v>
       </c>
       <c r="C2" s="37" t="s">
-        <v>38</v>
+        <v>77</v>
       </c>
       <c r="D2" s="37" t="s">
-        <v>39</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.3">
@@ -2677,11 +2616,11 @@
         <v>1</v>
       </c>
       <c r="B3" s="39" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="C3" s="40"/>
       <c r="D3" s="41" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.6" thickBot="1">
@@ -2689,11 +2628,11 @@
         <v>2</v>
       </c>
       <c r="B4" s="43" t="s">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="C4" s="44"/>
       <c r="D4" s="45" t="s">
-        <v>41</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.6" thickBot="1">
@@ -2701,11 +2640,11 @@
         <v>3</v>
       </c>
       <c r="B5" s="43" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="C5" s="44"/>
       <c r="D5" s="45" t="s">
-        <v>41</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="49" customFormat="1" ht="15.6" thickBot="1">
@@ -2715,25 +2654,25 @@
       <c r="D6" s="48"/>
     </row>
     <row r="7" spans="1:4" s="49" customFormat="1" ht="16.5" thickBot="1">
-      <c r="A7" s="82" t="s">
-        <v>42</v>
-      </c>
-      <c r="B7" s="83"/>
-      <c r="C7" s="83"/>
-      <c r="D7" s="84"/>
+      <c r="A7" s="80" t="s">
+        <v>83</v>
+      </c>
+      <c r="B7" s="81"/>
+      <c r="C7" s="81"/>
+      <c r="D7" s="82"/>
     </row>
     <row r="8" spans="1:4" s="49" customFormat="1" ht="15.6" thickBot="1">
       <c r="A8" s="50" t="s">
-        <v>104</v>
+        <v>55</v>
       </c>
       <c r="B8" s="51" t="s">
-        <v>105</v>
+        <v>56</v>
       </c>
       <c r="C8" s="51" t="s">
-        <v>38</v>
+        <v>77</v>
       </c>
       <c r="D8" s="51" t="s">
-        <v>106</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.3">
@@ -2741,7 +2680,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="53" t="s">
-        <v>43</v>
+        <v>85</v>
       </c>
       <c r="C9" s="54"/>
       <c r="D9" s="55"/>
@@ -2751,7 +2690,7 @@
         <v>4</v>
       </c>
       <c r="B10" s="39" t="s">
-        <v>44</v>
+        <v>86</v>
       </c>
       <c r="C10" s="56"/>
       <c r="D10" s="57"/>
@@ -2761,7 +2700,7 @@
         <v>5</v>
       </c>
       <c r="B11" s="39" t="s">
-        <v>45</v>
+        <v>87</v>
       </c>
       <c r="C11" s="56"/>
       <c r="D11" s="57"/>
@@ -2771,7 +2710,7 @@
         <v>6</v>
       </c>
       <c r="B12" s="39" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="C12" s="56"/>
       <c r="D12" s="57"/>
@@ -2781,7 +2720,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="39" t="s">
-        <v>47</v>
+        <v>89</v>
       </c>
       <c r="C13" s="56"/>
       <c r="D13" s="57"/>
@@ -2791,7 +2730,7 @@
         <v>8</v>
       </c>
       <c r="B14" s="39" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="C14" s="56"/>
       <c r="D14" s="57"/>
@@ -2801,7 +2740,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="56" t="s">
-        <v>49</v>
+        <v>91</v>
       </c>
       <c r="C15" s="56"/>
       <c r="D15" s="57"/>
@@ -2811,7 +2750,7 @@
         <v>10</v>
       </c>
       <c r="B16" s="39" t="s">
-        <v>50</v>
+        <v>92</v>
       </c>
       <c r="C16" s="56"/>
       <c r="D16" s="57"/>
@@ -2821,11 +2760,11 @@
         <v>11</v>
       </c>
       <c r="B17" s="39" t="s">
-        <v>51</v>
+        <v>93</v>
       </c>
       <c r="C17" s="56"/>
       <c r="D17" s="57" t="s">
-        <v>52</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15.3">
@@ -2833,7 +2772,7 @@
         <v>12</v>
       </c>
       <c r="B18" s="39" t="s">
-        <v>53</v>
+        <v>94</v>
       </c>
       <c r="C18" s="56"/>
       <c r="D18" s="57"/>
@@ -2843,7 +2782,7 @@
         <v>13</v>
       </c>
       <c r="B19" s="39" t="s">
-        <v>54</v>
+        <v>95</v>
       </c>
       <c r="C19" s="56"/>
       <c r="D19" s="57"/>
@@ -2853,7 +2792,7 @@
         <v>14</v>
       </c>
       <c r="B20" s="39" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="C20" s="56"/>
       <c r="D20" s="57"/>
@@ -2863,7 +2802,7 @@
         <v>15</v>
       </c>
       <c r="B21" s="39" t="s">
-        <v>56</v>
+        <v>97</v>
       </c>
       <c r="C21" s="56"/>
       <c r="D21" s="57"/>
@@ -2873,7 +2812,7 @@
         <v>16</v>
       </c>
       <c r="B22" s="43" t="s">
-        <v>57</v>
+        <v>98</v>
       </c>
       <c r="C22" s="58"/>
       <c r="D22" s="59"/>
@@ -2882,25 +2821,25 @@
       <c r="A23" s="60"/>
     </row>
     <row r="24" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A24" s="85" t="s">
-        <v>58</v>
-      </c>
-      <c r="B24" s="86"/>
-      <c r="C24" s="86"/>
-      <c r="D24" s="87"/>
+      <c r="A24" s="83" t="s">
+        <v>100</v>
+      </c>
+      <c r="B24" s="84"/>
+      <c r="C24" s="84"/>
+      <c r="D24" s="85"/>
     </row>
     <row r="25" spans="1:4" ht="15.6" thickBot="1">
       <c r="A25" s="61" t="s">
-        <v>104</v>
+        <v>55</v>
       </c>
       <c r="B25" s="62" t="s">
-        <v>105</v>
+        <v>56</v>
       </c>
       <c r="C25" s="62" t="s">
-        <v>38</v>
+        <v>77</v>
       </c>
       <c r="D25" s="62" t="s">
-        <v>39</v>
+        <v>84</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="14.7" thickBot="1">
@@ -2908,11 +2847,11 @@
         <v>17</v>
       </c>
       <c r="B26" s="63" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="C26" s="64"/>
       <c r="D26" s="65" t="s">
-        <v>60</v>
+        <v>82</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="14.7" thickBot="1">
@@ -2920,11 +2859,11 @@
         <v>18</v>
       </c>
       <c r="B27" s="63" t="s">
-        <v>61</v>
+        <v>101</v>
       </c>
       <c r="C27" s="40"/>
       <c r="D27" s="41" t="s">
-        <v>41</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="14.4">
@@ -2932,23 +2871,23 @@
         <v>19</v>
       </c>
       <c r="B28" s="63" t="s">
-        <v>62</v>
+        <v>102</v>
       </c>
       <c r="C28" s="66"/>
-      <c r="D28" s="67" t="s">
-        <v>63</v>
+      <c r="D28" s="87" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="14.7" thickBot="1">
       <c r="A29" s="38">
         <v>20</v>
       </c>
-      <c r="B29" s="68" t="s">
-        <v>64</v>
-      </c>
-      <c r="C29" s="69"/>
-      <c r="D29" s="70" t="s">
-        <v>63</v>
+      <c r="B29" s="67" t="s">
+        <v>103</v>
+      </c>
+      <c r="C29" s="68"/>
+      <c r="D29" s="88" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -2957,7 +2896,7 @@
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A24:D24"/>
   </mergeCells>
-  <phoneticPr fontId="34" type="noConversion"/>
+  <phoneticPr fontId="35" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C9:C22 C26:C29 C3:C5" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"Y,N"</formula1>
@@ -2983,54 +2922,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="88" t="s">
-        <v>21</v>
-      </c>
-      <c r="B1" s="88" t="s">
-        <v>100</v>
-      </c>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88" t="s">
-        <v>101</v>
+      <c r="A1" s="86" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="86" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="86"/>
+      <c r="D1" s="86" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="88"/>
+      <c r="A2" s="86"/>
       <c r="B2" s="16" t="s">
-        <v>22</v>
+        <v>68</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="88"/>
+        <v>67</v>
+      </c>
+      <c r="D2" s="86"/>
     </row>
     <row r="3" spans="1:4" ht="15">
       <c r="A3" s="17" t="s">
-        <v>70</v>
+        <v>24</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D3" s="19"/>
     </row>
     <row r="4" spans="1:4" ht="15">
       <c r="A4" s="17" t="s">
-        <v>71</v>
+        <v>25</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D4" s="19"/>
     </row>
     <row r="5" spans="1:4" ht="15">
       <c r="A5" s="21" t="s">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="B5" s="22"/>
       <c r="C5" s="22"/>
@@ -3038,19 +2977,19 @@
     </row>
     <row r="6" spans="1:4" ht="15">
       <c r="A6" s="23" t="s">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="B6" s="22"/>
       <c r="C6" s="22" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>27</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15">
       <c r="A7" s="21" t="s">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="B7" s="24"/>
       <c r="C7" s="24"/>
@@ -3058,39 +2997,39 @@
     </row>
     <row r="8" spans="1:4" ht="15">
       <c r="A8" s="23" t="s">
-        <v>28</v>
+        <v>72</v>
       </c>
       <c r="B8" s="25"/>
       <c r="C8" s="25" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D8" s="19"/>
     </row>
     <row r="9" spans="1:4" ht="15">
       <c r="A9" s="26" t="s">
-        <v>75</v>
+        <v>29</v>
       </c>
       <c r="B9" s="25"/>
       <c r="C9" s="25" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>30</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15">
       <c r="A10" s="23" t="s">
-        <v>76</v>
+        <v>30</v>
       </c>
       <c r="B10" s="25"/>
       <c r="C10" s="25" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D10" s="19"/>
     </row>
     <row r="11" spans="1:4" ht="15">
       <c r="A11" s="21" t="s">
-        <v>77</v>
+        <v>31</v>
       </c>
       <c r="B11" s="25"/>
       <c r="C11" s="25"/>
@@ -3098,29 +3037,29 @@
     </row>
     <row r="12" spans="1:4" ht="15">
       <c r="A12" s="23" t="s">
-        <v>13</v>
+        <v>74</v>
       </c>
       <c r="B12" s="25"/>
       <c r="C12" s="25" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D12" s="19"/>
     </row>
     <row r="13" spans="1:4" ht="15">
       <c r="A13" s="17" t="s">
-        <v>78</v>
+        <v>32</v>
       </c>
       <c r="B13" s="25" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D13" s="19"/>
     </row>
     <row r="14" spans="1:4" ht="15">
       <c r="A14" s="21" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="B14" s="25"/>
       <c r="C14" s="25"/>
@@ -3128,17 +3067,17 @@
     </row>
     <row r="15" spans="1:4" ht="15">
       <c r="A15" s="23" t="s">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="B15" s="25"/>
       <c r="C15" s="25" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D15" s="19"/>
     </row>
     <row r="16" spans="1:4" ht="15">
       <c r="A16" s="21" t="s">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="B16" s="25"/>
       <c r="C16" s="25"/>
@@ -3146,27 +3085,27 @@
     </row>
     <row r="17" spans="1:4" ht="15">
       <c r="A17" s="23" t="s">
-        <v>82</v>
+        <v>36</v>
       </c>
       <c r="B17" s="25"/>
       <c r="C17" s="25" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D17" s="19"/>
     </row>
     <row r="18" spans="1:4" ht="15">
       <c r="A18" s="23" t="s">
-        <v>83</v>
+        <v>37</v>
       </c>
       <c r="B18" s="25"/>
       <c r="C18" s="25" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D18" s="19"/>
     </row>
     <row r="19" spans="1:4" ht="15">
       <c r="A19" s="21" t="s">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="B19" s="25"/>
       <c r="C19" s="25"/>
@@ -3174,27 +3113,27 @@
     </row>
     <row r="20" spans="1:4" ht="15">
       <c r="A20" s="23" t="s">
-        <v>85</v>
+        <v>39</v>
       </c>
       <c r="B20" s="25"/>
       <c r="C20" s="25" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D20" s="19"/>
     </row>
     <row r="21" spans="1:4" ht="15">
       <c r="A21" s="26" t="s">
-        <v>86</v>
+        <v>40</v>
       </c>
       <c r="B21" s="25"/>
       <c r="C21" s="25" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="D21" s="19"/>
     </row>
     <row r="22" spans="1:4" ht="15">
       <c r="A22" s="21" t="s">
-        <v>87</v>
+        <v>41</v>
       </c>
       <c r="B22" s="25"/>
       <c r="C22" s="25"/>
@@ -3202,7 +3141,7 @@
     </row>
     <row r="23" spans="1:4" ht="15">
       <c r="A23" s="21" t="s">
-        <v>88</v>
+        <v>42</v>
       </c>
       <c r="B23" s="25"/>
       <c r="C23" s="25"/>
@@ -3210,7 +3149,7 @@
     </row>
     <row r="24" spans="1:4" ht="15">
       <c r="A24" s="21" t="s">
-        <v>89</v>
+        <v>43</v>
       </c>
       <c r="B24" s="25"/>
       <c r="C24" s="25"/>
@@ -3218,7 +3157,7 @@
     </row>
     <row r="25" spans="1:4" ht="15">
       <c r="A25" s="21" t="s">
-        <v>11</v>
+        <v>73</v>
       </c>
       <c r="B25" s="25"/>
       <c r="C25" s="25"/>
@@ -3226,7 +3165,7 @@
     </row>
     <row r="26" spans="1:4" ht="15">
       <c r="A26" s="21" t="s">
-        <v>90</v>
+        <v>44</v>
       </c>
       <c r="B26" s="25"/>
       <c r="C26" s="25"/>
@@ -3234,7 +3173,7 @@
     </row>
     <row r="27" spans="1:4" ht="15">
       <c r="A27" s="21" t="s">
-        <v>91</v>
+        <v>45</v>
       </c>
       <c r="B27" s="25"/>
       <c r="C27" s="25"/>
@@ -3242,27 +3181,27 @@
     </row>
     <row r="28" spans="1:4" ht="15">
       <c r="A28" s="23" t="s">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="B28" s="25"/>
       <c r="C28" s="25" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D28" s="19"/>
     </row>
     <row r="29" spans="1:4" ht="15">
       <c r="A29" s="23" t="s">
-        <v>92</v>
+        <v>46</v>
       </c>
       <c r="B29" s="25"/>
       <c r="C29" s="25" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D29" s="19"/>
     </row>
     <row r="30" spans="1:4" ht="15">
       <c r="A30" s="21" t="s">
-        <v>93</v>
+        <v>47</v>
       </c>
       <c r="B30" s="25"/>
       <c r="C30" s="25"/>
@@ -3270,7 +3209,7 @@
     </row>
     <row r="31" spans="1:4" ht="15">
       <c r="A31" s="21" t="s">
-        <v>94</v>
+        <v>48</v>
       </c>
       <c r="B31" s="25"/>
       <c r="C31" s="25"/>
@@ -3278,7 +3217,7 @@
     </row>
     <row r="32" spans="1:4" ht="15">
       <c r="A32" s="21" t="s">
-        <v>95</v>
+        <v>49</v>
       </c>
       <c r="B32" s="25"/>
       <c r="C32" s="25"/>
@@ -3286,7 +3225,7 @@
     </row>
     <row r="33" spans="1:4" ht="15">
       <c r="A33" s="21" t="s">
-        <v>96</v>
+        <v>50</v>
       </c>
       <c r="B33" s="25"/>
       <c r="C33" s="25"/>
@@ -3294,7 +3233,7 @@
     </row>
     <row r="34" spans="1:4" ht="15">
       <c r="A34" s="21" t="s">
-        <v>97</v>
+        <v>51</v>
       </c>
       <c r="B34" s="25"/>
       <c r="C34" s="25"/>
@@ -3302,7 +3241,7 @@
     </row>
     <row r="35" spans="1:4" ht="15">
       <c r="A35" s="21" t="s">
-        <v>98</v>
+        <v>52</v>
       </c>
       <c r="B35" s="25"/>
       <c r="C35" s="25"/>
@@ -3310,44 +3249,44 @@
     </row>
     <row r="36" spans="1:4" ht="15">
       <c r="A36" s="28" t="s">
-        <v>99</v>
+        <v>53</v>
       </c>
       <c r="B36" s="29"/>
       <c r="C36" s="29" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D36" s="19"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="30" t="s">
-        <v>102</v>
+        <v>54</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="15.3">
       <c r="A40" s="31"/>
       <c r="B40" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="C40" s="32" t="s">
-        <v>103</v>
+        <v>68</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="15.3">
       <c r="A41" s="33"/>
       <c r="B41" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="C41" s="32" t="s">
-        <v>23</v>
+        <v>67</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="15.3">
       <c r="A42" s="34"/>
       <c r="B42" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="C42" s="32" t="s">
-        <v>36</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -3356,7 +3295,7 @@
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="D1:D2"/>
   </mergeCells>
-  <phoneticPr fontId="34" type="noConversion"/>
+  <phoneticPr fontId="35" type="noConversion"/>
   <conditionalFormatting sqref="C7">
     <cfRule type="expression" dxfId="1" priority="2">
       <formula>"If(blnBinNo=""True"")"</formula>

</xml_diff>